<commit_message>
Verify full-period short-no-roll results and update thesis workbook
</commit_message>
<xml_diff>
--- a/outputs/thesis-system-20261016/deliverables/ESA_thesis_results.xlsx
+++ b/outputs/thesis-system-20261016/deliverables/ESA_thesis_results.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thesis results" sheetId="1" r:id="Rdd0d856c552f41a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thesis results" sheetId="1" r:id="R581d52b719be4215"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,6 +24,20 @@
       <x:text>
         <x:r>
           <x:t>Source: ESA-ADB, long-baseline results, 24 September 2026; source commit 523b0a4. Pooled and all annual metrics independently replayed from the original prediction mask and raw annotation IDs on 16 October 2026. https://github.com/kamyarfaz/ESA-ADB/blob/523b0a4/docs/research/long-baseline-results-2026-09-24.md</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A10" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>Source: docs/research/full-short-no-roll-results-2026-10-16.md and tables/full-short-no-roll-2026-10-16/verified_results.csv. All annual and pooled metrics independently replayed from saved predictions and raw annotation IDs on 16 October 2026.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A22" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>Source: docs/research/full-short-no-roll-results-2026-10-16.md and tables/full-short-no-roll-2026-10-16/verified_results.csv. All annual and pooled metrics independently replayed from saved predictions and raw annotation IDs on 16 October 2026.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -443,7 +457,7 @@
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>Shared budget: 40 epochs, all nominal training windows, batch 64. One planned run per technique, seed 42.</x:v>
+        <x:v>Shared budget: 40 epochs, all nominal training windows, batch 64. One completed run per technique, seed 42.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -454,7 +468,7 @@
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>System evaluation includes Anomaly and Rare Event IDs from all 76 channels. Only the baseline run is complete.</x:v>
+        <x:v>System evaluation includes Anomaly and Rare Event IDs from all 76 channels. Both runs are complete and verified.</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -537,20 +551,21 @@
       <x:c r="B10" s="16" t="str">
         <x:v>40–47</x:v>
       </x:c>
-      <x:c r="C10" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="D10" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E10" s="18" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="F10" s="20" t="str">
-        <x:v>Pending</x:v>
+      <x:c r="C10" s="17" t="n">
+        <x:v>0.9793058582615488</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="n">
+        <x:v>0.5274725274725275</x:v>
+      </x:c>
+      <x:c r="E10" s="18" t="n">
+        <x:v>0.0002919363580021761</x:v>
+      </x:c>
+      <x:c r="F10" s="20" t="n">
+        <x:f>IF(0.25*C10+D10=0,0,1.25*C10*D10/(0.25*C10+D10))</x:f>
+        <x:v>0.8360701968268796</x:v>
       </x:c>
       <x:c r="G10" s="16" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
@@ -702,20 +717,21 @@
       <x:c r="B22" s="22" t="n">
         <x:v>2007</x:v>
       </x:c>
-      <x:c r="C22" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="D22" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E22" s="18" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="F22" s="17" t="str">
-        <x:v>Pending</x:v>
+      <x:c r="C22" s="17" t="n">
+        <x:v>0.9995390140067242</x:v>
+      </x:c>
+      <x:c r="D22" s="17" t="n">
+        <x:v>0.6875</x:v>
+      </x:c>
+      <x:c r="E22" s="18" t="n">
+        <x:v>0.0004609859932758198</x:v>
+      </x:c>
+      <x:c r="F22" s="17" t="n">
+        <x:f>IF(0.25*C22+D22=0,0,1.25*C22*D22/(0.25*C22+D22))</x:f>
+        <x:v>0.916356743539128</x:v>
       </x:c>
       <x:c r="G22" s="16" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="28" customHeight="1">
@@ -749,20 +765,21 @@
       <x:c r="B24" s="22" t="n">
         <x:v>2008</x:v>
       </x:c>
-      <x:c r="C24" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="D24" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E24" s="18" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="F24" s="17" t="str">
-        <x:v>Pending</x:v>
+      <x:c r="C24" s="17" t="n">
+        <x:v>0.999508119418822</x:v>
+      </x:c>
+      <x:c r="D24" s="17" t="n">
+        <x:v>0.5384615384615384</x:v>
+      </x:c>
+      <x:c r="E24" s="18" t="n">
+        <x:v>0.0004918805811779947</x:v>
+      </x:c>
+      <x:c r="F24" s="17" t="n">
+        <x:f>IF(0.25*C24+D24=0,0,1.25*C24*D24/(0.25*C24+D24))</x:f>
+        <x:v>0.8533717322059889</x:v>
       </x:c>
       <x:c r="G24" s="16" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
@@ -796,20 +813,21 @@
       <x:c r="B26" s="22" t="n">
         <x:v>2009</x:v>
       </x:c>
-      <x:c r="C26" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="D26" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E26" s="18" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="F26" s="17" t="str">
-        <x:v>Pending</x:v>
+      <x:c r="C26" s="17" t="n">
+        <x:v>0.9995740169758751</x:v>
+      </x:c>
+      <x:c r="D26" s="17" t="n">
+        <x:v>0.5833333333333334</x:v>
+      </x:c>
+      <x:c r="E26" s="18" t="n">
+        <x:v>0.0004259830241248874</x:v>
+      </x:c>
+      <x:c r="F26" s="17" t="n">
+        <x:f>IF(0.25*C26+D26=0,0,1.25*C26*D26/(0.25*C26+D26))</x:f>
+        <x:v>0.8747390520499043</x:v>
       </x:c>
       <x:c r="G26" s="16" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="28" customHeight="1">
@@ -843,20 +861,21 @@
       <x:c r="B28" s="22" t="n">
         <x:v>2010</x:v>
       </x:c>
-      <x:c r="C28" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="D28" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E28" s="18" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="F28" s="17" t="str">
-        <x:v>Pending</x:v>
+      <x:c r="C28" s="17" t="n">
+        <x:v>0.9998081763526087</x:v>
+      </x:c>
+      <x:c r="D28" s="17" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E28" s="18" t="n">
+        <x:v>0.0001918236473913426</x:v>
+      </x:c>
+      <x:c r="F28" s="17" t="n">
+        <x:f>IF(0.25*C28+D28=0,0,1.25*C28*D28/(0.25*C28+D28))</x:f>
+        <x:v>0.624940049360215</x:v>
       </x:c>
       <x:c r="G28" s="16" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="28" customHeight="1">
@@ -890,20 +909,21 @@
       <x:c r="B30" s="22" t="n">
         <x:v>2011</x:v>
       </x:c>
-      <x:c r="C30" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="D30" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E30" s="18" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="F30" s="17" t="str">
-        <x:v>Pending</x:v>
+      <x:c r="C30" s="17" t="n">
+        <x:v>0.9998584247339305</x:v>
+      </x:c>
+      <x:c r="D30" s="17" t="n">
+        <x:v>0.5333333333333333</x:v>
+      </x:c>
+      <x:c r="E30" s="18" t="n">
+        <x:v>0.00014157526606950466</x:v>
+      </x:c>
+      <x:c r="F30" s="17" t="n">
+        <x:f>IF(0.25*C30+D30=0,0,1.25*C30*D30/(0.25*C30+D30))</x:f>
+        <x:v>0.850981790616141</x:v>
       </x:c>
       <x:c r="G30" s="16" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
@@ -937,20 +957,21 @@
       <x:c r="B32" s="22" t="n">
         <x:v>2012</x:v>
       </x:c>
-      <x:c r="C32" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="D32" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E32" s="18" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="F32" s="17" t="str">
-        <x:v>Pending</x:v>
+      <x:c r="C32" s="17" t="n">
+        <x:v>0.7999153173230444</x:v>
+      </x:c>
+      <x:c r="D32" s="17" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="E32" s="18" t="n">
+        <x:v>0.00010585334619450659</x:v>
+      </x:c>
+      <x:c r="F32" s="17" t="n">
+        <x:f>IF(0.25*C32+D32=0,0,1.25*C32*D32/(0.25*C32+D32))</x:f>
+        <x:v>0.6666196190749765</x:v>
       </x:c>
       <x:c r="G32" s="16" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
@@ -984,20 +1005,21 @@
       <x:c r="B34" s="22" t="n">
         <x:v>2013</x:v>
       </x:c>
-      <x:c r="C34" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="D34" s="17" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="E34" s="18" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="F34" s="17" t="str">
-        <x:v>Pending</x:v>
+      <x:c r="C34" s="17" t="n">
+        <x:v>0.9997639198660909</x:v>
+      </x:c>
+      <x:c r="D34" s="17" t="n">
+        <x:v>0.5714285714285714</x:v>
+      </x:c>
+      <x:c r="E34" s="18" t="n">
+        <x:v>0.0002360801339090779</x:v>
+      </x:c>
+      <x:c r="F34" s="17" t="n">
+        <x:f>IF(0.25*C34+D34=0,0,1.25*C34*D34/(0.25*C34+D34))</x:f>
+        <x:v>0.8694223987311318</x:v>
       </x:c>
       <x:c r="G34" s="16" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
@@ -1026,6 +1048,6 @@
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="In progress"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9729983fecac4836"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bdba4d802914153"/>
 </x:worksheet>
 </file>
</xml_diff>